<commit_message>
Update quick self-assessment: scenario-targeted survey (Agentic/RAG/Standalone) and 3-sheet Excel workbook
</commit_message>
<xml_diff>
--- a/specification/AITBM_Quick_Assessment.xlsx
+++ b/specification/AITBM_Quick_Assessment.xlsx
@@ -7,8 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Assessment" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engine" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agentic" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agentic Engine" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RAG" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RAG Engine" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standalone" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standalone Engine" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,7 +34,7 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="001F3864"/>
-      <sz val="16"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -109,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -130,6 +134,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -495,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -507,14 +512,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AITBM — Quick AI Risk Self-Assessment</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
+          <t>AITBM — Quick AI Risk Self-Assessment — Agentic / MCP</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Answer Yes or No in column C. Your Effective Risk Score (ERS) updates automatically. Educational estimate; see the AITBM Framework Specification for assessments of record.</t>
+          <t>Scenario: Agentic / MCP. Answer Yes or No in column C; the Effective Risk Score (ERS) updates automatically. The Agentic / RAG / Standalone tabs each carry questions tailored to that architecture. Educational estimate; see the AITBM Framework Specification for assessments of record.</t>
         </is>
       </c>
     </row>
@@ -526,7 +531,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>About your AI system — A few questions about what the system does and where it runs.</t>
+          <t>About your system — A few questions about what your AI agent does and where it runs.</t>
         </is>
       </c>
       <c r="C4" s="3" t="n"/>
@@ -535,7 +540,7 @@
     <row r="5" ht="28" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Is it an AI agent — can it call tools, take actions, or operate other systems (not just return text)?</t>
+          <t>Can the agent take actions or make decisions on its own, without a person approving each step?</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -547,7 +552,7 @@
     <row r="6" ht="28" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Does it use retrieval / RAG — pulling from documents or a knowledge base to answer?</t>
+          <t>Can it reach untrusted input — the public internet, external tools/APIs, or third-party content?</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -559,7 +564,7 @@
     <row r="7" ht="28" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Can it act without a person approving each action or decision?</t>
+          <t>Could a wrong action cause serious harm — money moved, data changed, safety, or many systems affected?</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -571,7 +576,7 @@
     <row r="8" ht="28" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Can the public or untrusted users send input to it (internet-facing, public API, external content)?</t>
+          <t>Would a bad action be slow or hard to undo (no kill-switch, no quick rollback, vendor lock-in)?</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -580,52 +585,60 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Could a failure or compromise cause serious harm — financial loss, safety, legal/regulatory, or many users/systems?</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="28" customHeight="1">
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Would a discovered problem be slow or hard to fix (needs retraining, vendor dependency, no quick rollback)?</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Safeguards in place — Answer Yes only for protections you have actually implemented.</t>
         </is>
       </c>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="C10" s="3" t="n"/>
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Points you could save</t>
         </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Is the agent restricted to least-privilege — limited actions, tools, and systems it can reach?</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D11" s="6">
+        <f>IF('Agentic'!$C$11="Yes","",ROUND('Agentic Engine'!B49,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Does a human review or approve the agent's high-impact actions before they take effect?</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D12" s="6">
+        <f>IF('Agentic'!$C$12="Yes","",ROUND('Agentic Engine'!B50,1))</f>
+        <v/>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Do you filter and validate both the inputs users send and the outputs the model returns?</t>
+          <t>Do you verify each agent's identity and monitor agent behavior for anomalies?</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -634,14 +647,14 @@
         </is>
       </c>
       <c r="D13" s="6">
-        <f>IF('Quick Assessment'!$C$13="Yes","",ROUND(Engine!B55,1))</f>
+        <f>IF('Agentic'!$C$13="Yes","",ROUND('Agentic Engine'!B51,1))</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Do you have real-time monitoring/detection for prompt injection, abuse, or abnormal behavior?</t>
+          <t>Do you control which tools/skills the agent may use, and route its calls through a vetted gateway?</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -650,14 +663,14 @@
         </is>
       </c>
       <c r="D14" s="6">
-        <f>IF('Quick Assessment'!$C$14="Yes","",ROUND(Engine!B56,1))</f>
+        <f>IF('Agentic'!$C$14="Yes","",ROUND('Agentic Engine'!B52,1))</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Have you tested the model against adversarial / manipulated inputs and hardened it?</t>
+          <t>Is the agent sandboxed and network-segmented away from sensitive systems?</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -666,14 +679,14 @@
         </is>
       </c>
       <c r="D15" s="6">
-        <f>IF('Quick Assessment'!$C$15="Yes","",ROUND(Engine!B57,1))</f>
+        <f>IF('Agentic'!$C$15="Yes","",ROUND('Agentic Engine'!B53,1))</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Does a human review or approve the AI's high-impact actions before they take effect?</t>
+          <t>Do you filter and validate both the inputs the agent receives and the outputs/actions it produces?</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -682,14 +695,14 @@
         </is>
       </c>
       <c r="D16" s="6">
-        <f>IF('Quick Assessment'!$C$16="Yes","",ROUND(Engine!B58,1))</f>
+        <f>IF('Agentic'!$C$16="Yes","",ROUND('Agentic Engine'!B54,1))</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Is the AI restricted to least-privilege — limited actions, tools, and systems it can reach?</t>
+          <t>Do you have real-time detection for prompt injection, tool abuse, or abnormal agent behavior?</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -698,14 +711,14 @@
         </is>
       </c>
       <c r="D17" s="6">
-        <f>IF('Quick Assessment'!$C$17="Yes","",ROUND(Engine!B59,1))</f>
+        <f>IF('Agentic'!$C$17="Yes","",ROUND('Agentic Engine'!B55,1))</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Do you verify each agent's identity and monitor agent behavior for anomalies?</t>
+          <t>Do you track the agent's tools/model/data provenance (inventory, lineage) and document expected behavior?</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -714,46 +727,28 @@
         </is>
       </c>
       <c r="D18" s="6">
-        <f>IF('Quick Assessment'!$C$18="Yes","",ROUND(Engine!B60,1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="28" customHeight="1">
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Is the AI isolated from sensitive systems and networks (sandboxing / segmentation)?</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D19" s="6">
-        <f>IF('Quick Assessment'!$C$19="Yes","",ROUND(Engine!B61,1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="28" customHeight="1">
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Do you detect and block leakage of sensitive or personal data in AI outputs?</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D20" s="6">
-        <f>IF('Quick Assessment'!$C$20="Yes","",ROUND(Engine!B62,1))</f>
-        <v/>
-      </c>
+        <f>IF('Agentic'!$C$18="Yes","",ROUND('Agentic Engine'!B56,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Evidence &amp; assurance — How well the system's security is documented and tested.</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n"/>
+      <c r="D20" s="3" t="n"/>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Do you track where your model and data came from (lineage / AIBOM) and document expected behavior?</t>
+          <t>Do you have an AIBOM / model card AND an inventory of the agent's tools and their sources?</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -761,102 +756,73 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D21" s="6">
-        <f>IF('Quick Assessment'!$C$21="Yes","",ROUND(Engine!B63,1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Evidence &amp; assurance — How well the system's security is documented and tested.</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="n"/>
-      <c r="D23" s="3" t="n"/>
-    </row>
-    <row r="24" ht="28" customHeight="1">
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Do you have a model card / AI bill of materials documenting model and data provenance?</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="28" customHeight="1">
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Have you run security testing / red-teaming on this system (beyond normal QA)?</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="28" customHeight="1">
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Was that testing recent (within ~12 months) and kept current?</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Have you red-teamed the agent (tool abuse, prompt injection, privilege escalation)?</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Was that testing recent (within ~12 months) and repeated after changes to tools or prompts?</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>RESULT</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n"/>
+      <c r="C26" s="3" t="n"/>
+      <c r="D26" s="3" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Effective Risk Score (ERS)</t>
+        </is>
+      </c>
+      <c r="C27" s="8">
+        <f>ROUND('Agentic Engine'!B46,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="C28">
+        <f>IF('Agentic Engine'!B46&gt;=9,"Critical",IF('Agentic Engine'!B46&gt;=7,"High",IF('Agentic Engine'!B46&gt;=5,"Moderate",IF('Agentic Engine'!B46&gt;=3,"Low-Moderate","Low"))))</f>
+        <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>RESULT</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="n"/>
-      <c r="C29" s="3" t="n"/>
-      <c r="D29" s="3" t="n"/>
-    </row>
-    <row r="30">
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>Effective Risk Score (ERS)</t>
-        </is>
-      </c>
-      <c r="C30" s="8">
-        <f>ROUND(Engine!B52,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>Severity</t>
-        </is>
-      </c>
-      <c r="C31">
-        <f>IF(Engine!B52&gt;=9,"Critical",IF(Engine!B52&gt;=7,"High",IF(Engine!B52&gt;=5,"Moderate",IF(Engine!B52&gt;=3,"Low-Moderate","Low"))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="9" t="inlineStr">
-        <is>
-          <t>Inferred architecture</t>
-        </is>
-      </c>
-      <c r="C32">
-        <f>Engine!B30</f>
-        <v/>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Agentic / MCP</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -865,7 +831,7 @@
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C5 C6 C7 C8 C9 C10 C13 C14 C15 C16 C17 C18 C19 C20 C21 C24 C25 C26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C5 C6 C7 C8 C11 C12 C13 C14 C15 C16 C17 C18 C21 C22 C23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -879,7 +845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -919,7 +885,7 @@
         <v>0.2</v>
       </c>
       <c r="D2">
-        <f>MAX(C2,IF('Quick Assessment'!$C$13="Yes",0.65,0),IF('Quick Assessment'!$C$14="Yes",0.75,0),IF('Quick Assessment'!$C$15="Yes",0.7,0))</f>
+        <f>MAX(C2,IF('Agentic'!$C$16="Yes",0.65,0),IF('Agentic'!$C$17="Yes",0.75,0))</f>
         <v/>
       </c>
     </row>
@@ -957,7 +923,7 @@
         <v>0.25</v>
       </c>
       <c r="D4">
-        <f>MAX(C4,IF('Quick Assessment'!$C$14="Yes",0.65,0),IF('Quick Assessment'!$C$21="Yes",0.7,0))</f>
+        <f>MAX(C4,IF('Agentic'!$C$17="Yes",0.65,0),IF('Agentic'!$C$18="Yes",0.7,0))</f>
         <v/>
       </c>
     </row>
@@ -976,7 +942,7 @@
         <v>0.15</v>
       </c>
       <c r="D5">
-        <f>MAX(C5,IF('Quick Assessment'!$C$14="Yes",0.55,0),IF('Quick Assessment'!$C$15="Yes",0.65,0),IF('Quick Assessment'!$C$21="Yes",0.7,0))</f>
+        <f>MAX(C5,IF('Agentic'!$C$14="Yes",0.55,0),IF('Agentic'!$C$17="Yes",0.55,0),IF('Agentic'!$C$18="Yes",0.7,0))</f>
         <v/>
       </c>
     </row>
@@ -1071,7 +1037,7 @@
         <v>0.5</v>
       </c>
       <c r="D10">
-        <f>MAX(C10,IF('Quick Assessment'!$C$21="Yes",0.6,0))</f>
+        <f>MAX(C10,IF('Agentic'!$C$18="Yes",0.6,0))</f>
         <v/>
       </c>
     </row>
@@ -1090,7 +1056,7 @@
         <v>0.3</v>
       </c>
       <c r="D11">
-        <f>MAX(C11,IF('Quick Assessment'!$C$13="Yes",0.7,0),IF('Quick Assessment'!$C$14="Yes",0.6,0),IF('Quick Assessment'!$C$21="Yes",0.75,0))</f>
+        <f>MAX(C11,IF('Agentic'!$C$16="Yes",0.7,0),IF('Agentic'!$C$17="Yes",0.6,0),IF('Agentic'!$C$18="Yes",0.75,0))</f>
         <v/>
       </c>
     </row>
@@ -1109,7 +1075,7 @@
         <v>0.4</v>
       </c>
       <c r="D12">
-        <f>MAX(C12,IF('Quick Assessment'!$C$14="Yes",0.65,0))</f>
+        <f>MAX(C12,IF('Agentic'!$C$17="Yes",0.65,0))</f>
         <v/>
       </c>
     </row>
@@ -1128,7 +1094,7 @@
         <v>0</v>
       </c>
       <c r="D13">
-        <f>MAX(C13,IF('Quick Assessment'!$C$21="Yes",0.8,0))</f>
+        <f>MAX(C13,IF('Agentic'!$C$18="Yes",0.8,0))</f>
         <v/>
       </c>
     </row>
@@ -1147,7 +1113,7 @@
         <v>0.25</v>
       </c>
       <c r="D14">
-        <f>MAX(C14,IF('Quick Assessment'!$C$13="Yes",0.6,0),IF('Quick Assessment'!$C$20="Yes",0.7,0))</f>
+        <f>MAX(C14,IF('Agentic'!$C$16="Yes",0.6,0))</f>
         <v/>
       </c>
     </row>
@@ -1185,7 +1151,7 @@
         <v>0.3</v>
       </c>
       <c r="D16">
-        <f>MAX(C16,IF('Quick Assessment'!$C$20="Yes",0.65,0),IF('Quick Assessment'!$C$21="Yes",0.7,0))</f>
+        <f>MAX(C16,IF('Agentic'!$C$18="Yes",0.7,0))</f>
         <v/>
       </c>
     </row>
@@ -1223,7 +1189,7 @@
         <v>0.1</v>
       </c>
       <c r="D18">
-        <f>MAX(C18,IF('Quick Assessment'!$C$16="Yes",0.75,0),IF('Quick Assessment'!$C$17="Yes",0.8,0),IF('Quick Assessment'!$C$18="Yes",0.75,0),IF('Quick Assessment'!$C$19="Yes",0.7,0),IF('Quick Assessment'!$C$21="Yes",0.6,0))</f>
+        <f>MAX(C18,IF('Agentic'!$C$11="Yes",0.8,0),IF('Agentic'!$C$12="Yes",0.75,0),IF('Agentic'!$C$13="Yes",0.75,0),IF('Agentic'!$C$14="Yes",0.65,0),IF('Agentic'!$C$15="Yes",0.7,0),IF('Agentic'!$C$18="Yes",0.6,0))</f>
         <v/>
       </c>
     </row>
@@ -1242,7 +1208,7 @@
         <v>0.15</v>
       </c>
       <c r="D19">
-        <f>MAX(C19,IF('Quick Assessment'!$C$16="Yes",0.7,0),IF('Quick Assessment'!$C$17="Yes",0.75,0),IF('Quick Assessment'!$C$18="Yes",0.7,0))</f>
+        <f>MAX(C19,IF('Agentic'!$C$11="Yes",0.75,0),IF('Agentic'!$C$12="Yes",0.7,0),IF('Agentic'!$C$13="Yes",0.7,0))</f>
         <v/>
       </c>
     </row>
@@ -1261,7 +1227,7 @@
         <v>0.1</v>
       </c>
       <c r="D20">
-        <f>MAX(C20,IF('Quick Assessment'!$C$13="Yes",0.75,0),IF('Quick Assessment'!$C$19="Yes",0.65,0),IF('Quick Assessment'!$C$20="Yes",0.7,0))</f>
+        <f>MAX(C20,IF('Agentic'!$C$15="Yes",0.65,0),IF('Agentic'!$C$16="Yes",0.75,0))</f>
         <v/>
       </c>
     </row>
@@ -1280,7 +1246,7 @@
         <v>0.2</v>
       </c>
       <c r="D21">
-        <f>MAX(C21,IF('Quick Assessment'!$C$19="Yes",0.6,0))</f>
+        <f>MAX(C21,IF('Agentic'!$C$14="Yes",0.55,0),IF('Agentic'!$C$15="Yes",0.6,0))</f>
         <v/>
       </c>
     </row>
@@ -1299,7 +1265,7 @@
         <v>0.2</v>
       </c>
       <c r="D22">
-        <f>MAX(C22,IF('Quick Assessment'!$C$17="Yes",0.7,0),IF('Quick Assessment'!$C$18="Yes",0.8,0))</f>
+        <f>MAX(C22,IF('Agentic'!$C$11="Yes",0.7,0),IF('Agentic'!$C$13="Yes",0.8,0))</f>
         <v/>
       </c>
     </row>
@@ -1368,326 +1334,2431 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>arch</t>
+          <t>IVP</t>
         </is>
       </c>
       <c r="B30">
-        <f>IF('Quick Assessment'!$C$5="Yes","agentic",IF('Quick Assessment'!$C$6="Yes","rag","standalone"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>w_Ro</t>
-        </is>
-      </c>
-      <c r="B31">
-        <f>IF(B30="agentic",0.15,IF(B30="rag",0.25,0.25))</f>
+        <f>0.15*B24+0.1*B25+0.15*B26+0.15*B27+0.45*B28</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>w_Fa</t>
+          <t>aa</t>
         </is>
       </c>
       <c r="B32">
-        <f>IF(B30="agentic",0.1,IF(B30="rag",0.1,0.2))</f>
+        <f>IF('Agentic'!$C$5="Yes",0.85,0.3)</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>w_Tr</t>
+          <t>as</t>
         </is>
       </c>
       <c r="B33">
-        <f>IF(B30="agentic",0.15,IF(B30="rag",0.15,0.2))</f>
+        <f>IF('Agentic'!$C$6="Yes",0.85,0.3)</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>w_Pr</t>
+          <t>cp</t>
         </is>
       </c>
       <c r="B34">
-        <f>IF(B30="agentic",0.15,IF(B30="rag",0.3,0.2))</f>
+        <f>IF('Agentic'!$C$7="Yes",0.85,0.3)</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>w_Cn</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="B35">
-        <f>IF(B30="agentic",0.45,IF(B30="rag",0.2,0.15))</f>
+        <f>IF('Agentic'!$C$8="Yes",0.85,0.3)</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>IVP</t>
+          <t>orp_avg</t>
         </is>
       </c>
       <c r="B36">
-        <f>B31*B24+B32*B25+B33*B26+B34*B27+B35*B28</f>
+        <f>AVERAGE(B32:B35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>n_elev</t>
+        </is>
+      </c>
+      <c r="B37">
+        <f>(IF(B32&gt;0.75,1,0)+IF(B33&gt;0.75,1,0)+IF(B34&gt;0.75,1,0)+IF(B35&gt;0.75,1,0))</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>aa</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B38">
-        <f>IF('Quick Assessment'!$C$7="Yes",0.85,0.3)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>as</t>
-        </is>
-      </c>
-      <c r="B39">
-        <f>IF('Quick Assessment'!$C$8="Yes",0.85,0.3)</f>
+        <f>MIN(1.75,MAX(0.75,-0.129+1.882*B36+0.05*B37))</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>cp</t>
+          <t>pc</t>
         </is>
       </c>
       <c r="B40">
-        <f>IF('Quick Assessment'!$C$9="Yes",0.85,0.3)</f>
+        <f>IF('Agentic'!$C$21="Yes",0.8,0.2)</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>ec</t>
         </is>
       </c>
       <c r="B41">
-        <f>IF('Quick Assessment'!$C$10="Yes",0.85,0.3)</f>
+        <f>IF('Agentic'!$C$22="Yes",0.8,0.2)</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>orp_avg</t>
+          <t>tf</t>
         </is>
       </c>
       <c r="B42">
-        <f>AVERAGE(B38:B41)</f>
+        <f>IF('Agentic'!$C$22="Yes",IF('Agentic'!$C$23="Yes",0.8,0.25),0.2)</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>n_elev</t>
+          <t>ACI</t>
         </is>
       </c>
       <c r="B43">
-        <f>(IF(B38&gt;0.75,1,0)+IF(B39&gt;0.75,1,0)+IF(B40&gt;0.75,1,0)+IF(B41&gt;0.75,1,0))</f>
+        <f>(MAX(B40,0.01)*MAX(B41,0.01)*MAX(B42,0.01))^(1/3)</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>aci_mod</t>
         </is>
       </c>
       <c r="B44">
-        <f>MIN(1.75,MAX(0.75,-0.129+1.882*B42+0.05*B43))</f>
+        <f>1.1-0.525*B43</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>pc</t>
+          <t>ERS</t>
         </is>
       </c>
       <c r="B46">
-        <f>IF('Quick Assessment'!$C$24="Yes",0.8,0.2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>ec</t>
-        </is>
-      </c>
-      <c r="B47">
-        <f>IF('Quick Assessment'!$C$25="Yes",0.8,0.2)</f>
+        <f>MIN(10,MAX(1.5,1.5+8.5*(1-B30)*B38*B44))</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>tf</t>
-        </is>
-      </c>
-      <c r="B48">
-        <f>IF('Quick Assessment'!$C$25="Yes",IF('Quick Assessment'!$C$26="Yes",0.8,0.25),0.2)</f>
-        <v/>
+          <t>points-you-could-save (per safeguard)</t>
+        </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ACI</t>
+          <t>s1</t>
         </is>
       </c>
       <c r="B49">
-        <f>(MAX(B46,0.01)*MAX(B47,0.01)*MAX(B48,0.01))^(1/3)</f>
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.15*((D2+D3+D4+D5)/4)+0.1*((D6+D7+D8+D9)/4)+0.15*((D10+D11+D12+D13)/4)+0.15*((D14+D15+D16+D17)/4)+0.45*((MAX(D18,0.8)+MAX(D19,0.75)+D20+D21+MAX(D22,0.7))/5))))*B38*B44)))</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>aci_mod</t>
+          <t>s2</t>
         </is>
       </c>
       <c r="B50">
-        <f>1.1-0.525*B49</f>
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.15*((D2+D3+D4+D5)/4)+0.1*((D6+D7+D8+D9)/4)+0.15*((D10+D11+D12+D13)/4)+0.15*((D14+D15+D16+D17)/4)+0.45*((MAX(D18,0.75)+MAX(D19,0.7)+D20+D21+D22)/5))))*B38*B44)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>s3</t>
+        </is>
+      </c>
+      <c r="B51">
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.15*((D2+D3+D4+D5)/4)+0.1*((D6+D7+D8+D9)/4)+0.15*((D10+D11+D12+D13)/4)+0.15*((D14+D15+D16+D17)/4)+0.45*((MAX(D18,0.75)+MAX(D19,0.7)+D20+D21+MAX(D22,0.8))/5))))*B38*B44)))</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ERS</t>
+          <t>s4</t>
         </is>
       </c>
       <c r="B52">
-        <f>MIN(10,MAX(1.5,1.5+8.5*(1-B36)*B44*B50))</f>
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.15*((D2+D3+D4+MAX(D5,0.55))/4)+0.1*((D6+D7+D8+D9)/4)+0.15*((D10+D11+D12+D13)/4)+0.15*((D14+D15+D16+D17)/4)+0.45*((MAX(D18,0.65)+D19+D20+MAX(D21,0.55)+D22)/5))))*B38*B44)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>s5</t>
+        </is>
+      </c>
+      <c r="B53">
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.15*((D2+D3+D4+D5)/4)+0.1*((D6+D7+D8+D9)/4)+0.15*((D10+D11+D12+D13)/4)+0.15*((D14+D15+D16+D17)/4)+0.45*((MAX(D18,0.7)+D19+MAX(D20,0.65)+MAX(D21,0.6)+D22)/5))))*B38*B44)))</f>
         <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>points-you-could-save (per safeguard)</t>
-        </is>
+          <t>s6</t>
+        </is>
+      </c>
+      <c r="B54">
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.15*((MAX(D2,0.65)+D3+D4+D5)/4)+0.1*((D6+D7+D8+D9)/4)+0.15*((D10+MAX(D11,0.7)+D12+D13)/4)+0.15*((MAX(D14,0.6)+D15+D16+D17)/4)+0.45*((D18+D19+MAX(D20,0.75)+D21+D22)/5))))*B38*B44)))</f>
+        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>q7</t>
+          <t>s7</t>
         </is>
       </c>
       <c r="B55">
-        <f>MAX(0,B52-MIN(10,MAX(1.5,1.5+8.5*(1-((B31*((MAX(D2,0.65)+D3+D4+D5)/4)+B32*((D6+D7+D8+D9)/4)+B33*((D10+MAX(D11,0.7)+D12+D13)/4)+B34*((MAX(D14,0.6)+D15+D16+D17)/4)+B35*((D18+D19+MAX(D20,0.75)+D21+D22)/5))))*B44*B50)))</f>
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.15*((MAX(D2,0.75)+D3+MAX(D4,0.65)+MAX(D5,0.55))/4)+0.1*((D6+D7+D8+D9)/4)+0.15*((D10+MAX(D11,0.6)+MAX(D12,0.65)+D13)/4)+0.15*((D14+D15+D16+D17)/4)+0.45*((D18+D19+D20+D21+D22)/5))))*B38*B44)))</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>q8</t>
+          <t>s8</t>
         </is>
       </c>
       <c r="B56">
-        <f>MAX(0,B52-MIN(10,MAX(1.5,1.5+8.5*(1-((B31*((MAX(D2,0.75)+D3+MAX(D4,0.65)+MAX(D5,0.55))/4)+B32*((D6+D7+D8+D9)/4)+B33*((D10+MAX(D11,0.6)+MAX(D12,0.65)+D13)/4)+B34*((D14+D15+D16+D17)/4)+B35*((D18+D19+D20+D21+D22)/5))))*B44*B50)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>q9</t>
-        </is>
-      </c>
-      <c r="B57">
-        <f>MAX(0,B52-MIN(10,MAX(1.5,1.5+8.5*(1-((B31*((MAX(D2,0.7)+D3+D4+MAX(D5,0.65))/4)+B32*((D6+D7+D8+D9)/4)+B33*((D10+D11+D12+D13)/4)+B34*((D14+D15+D16+D17)/4)+B35*((D18+D19+D20+D21+D22)/5))))*B44*B50)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>q10</t>
-        </is>
-      </c>
-      <c r="B58">
-        <f>MAX(0,B52-MIN(10,MAX(1.5,1.5+8.5*(1-((B31*((D2+D3+D4+D5)/4)+B32*((D6+D7+D8+D9)/4)+B33*((D10+D11+D12+D13)/4)+B34*((D14+D15+D16+D17)/4)+B35*((MAX(D18,0.75)+MAX(D19,0.7)+D20+D21+D22)/5))))*B44*B50)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>q11</t>
-        </is>
-      </c>
-      <c r="B59">
-        <f>MAX(0,B52-MIN(10,MAX(1.5,1.5+8.5*(1-((B31*((D2+D3+D4+D5)/4)+B32*((D6+D7+D8+D9)/4)+B33*((D10+D11+D12+D13)/4)+B34*((D14+D15+D16+D17)/4)+B35*((MAX(D18,0.8)+MAX(D19,0.75)+D20+D21+MAX(D22,0.7))/5))))*B44*B50)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>q12</t>
-        </is>
-      </c>
-      <c r="B60">
-        <f>MAX(0,B52-MIN(10,MAX(1.5,1.5+8.5*(1-((B31*((D2+D3+D4+D5)/4)+B32*((D6+D7+D8+D9)/4)+B33*((D10+D11+D12+D13)/4)+B34*((D14+D15+D16+D17)/4)+B35*((MAX(D18,0.75)+MAX(D19,0.7)+D20+D21+MAX(D22,0.8))/5))))*B44*B50)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>q13</t>
-        </is>
-      </c>
-      <c r="B61">
-        <f>MAX(0,B52-MIN(10,MAX(1.5,1.5+8.5*(1-((B31*((D2+D3+D4+D5)/4)+B32*((D6+D7+D8+D9)/4)+B33*((D10+D11+D12+D13)/4)+B34*((D14+D15+D16+D17)/4)+B35*((MAX(D18,0.7)+D19+MAX(D20,0.65)+MAX(D21,0.6)+D22)/5))))*B44*B50)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>q14</t>
-        </is>
-      </c>
-      <c r="B62">
-        <f>MAX(0,B52-MIN(10,MAX(1.5,1.5+8.5*(1-((B31*((D2+D3+D4+D5)/4)+B32*((D6+D7+D8+D9)/4)+B33*((D10+D11+D12+D13)/4)+B34*((MAX(D14,0.7)+D15+MAX(D16,0.65)+D17)/4)+B35*((D18+D19+MAX(D20,0.7)+D21+D22)/5))))*B44*B50)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>q15</t>
-        </is>
-      </c>
-      <c r="B63">
-        <f>MAX(0,B52-MIN(10,MAX(1.5,1.5+8.5*(1-((B31*((D2+D3+MAX(D4,0.7)+MAX(D5,0.7))/4)+B32*((D6+D7+D8+D9)/4)+B33*((MAX(D10,0.6)+MAX(D11,0.75)+D12+MAX(D13,0.8))/4)+B34*((D14+D15+MAX(D16,0.7)+D17)/4)+B35*((MAX(D18,0.6)+D19+D20+D21+D22)/5))))*B44*B50)))</f>
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.15*((D2+D3+MAX(D4,0.7)+MAX(D5,0.7))/4)+0.1*((D6+D7+D8+D9)/4)+0.15*((MAX(D10,0.6)+MAX(D11,0.75)+D12+MAX(D13,0.8))/4)+0.15*((D14+D15+MAX(D16,0.7)+D17)/4)+0.45*((MAX(D18,0.6)+D19+D20+D21+D22)/5))))*B38*B44)))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>AITBM — Quick AI Risk Self-Assessment — RAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Scenario: RAG. Answer Yes or No in column C; the Effective Risk Score (ERS) updates automatically. The Agentic / RAG / Standalone tabs each carry questions tailored to that architecture. Educational estimate; see the AITBM Framework Specification for assessments of record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>About your system — A few questions about your retrieval-augmented (RAG) system and its data.</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Does the system act on retrieved content automatically (e.g., trigger actions), rather than only answering?</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Can untrusted or externally-sourced documents enter the knowledge base, or be retrieved at query time?</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Could a wrong or poisoned answer cause serious harm (financial, legal, safety, or a wide audience)?</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Would correcting a bad answer be slow (re-indexing, re-embedding, vendor dependency, no quick fix)?</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Safeguards in place — Answer Yes only for protections you have actually implemented.</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n"/>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Points you could save</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Is your RAG pipeline secured — retrieved content validated and access-controlled before use?</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D11" s="6">
+        <f>IF('RAG'!$C$11="Yes","",ROUND('RAG Engine'!B49,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Do you detect and block leakage of sensitive or personal data in answers?</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D12" s="6">
+        <f>IF('RAG'!$C$12="Yes","",ROUND('RAG Engine'!B50,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Do you filter and validate both the user query and the generated answer?</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D13" s="6">
+        <f>IF('RAG'!$C$13="Yes","",ROUND('RAG Engine'!B51,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Do you detect indirect prompt injection carried inside retrieved documents?</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D14" s="6">
+        <f>IF('RAG'!$C$14="Yes","",ROUND('RAG Engine'!B52,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Do you resist data poisoning of the corpus or training data (vetting, adversarial hardening)?</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D15" s="6">
+        <f>IF('RAG'!$C$15="Yes","",ROUND('RAG Engine'!B53,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Do you track provenance/lineage of the model AND the knowledge-base sources?</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D16" s="6">
+        <f>IF('RAG'!$C$16="Yes","",ROUND('RAG Engine'!B54,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Are the vector store, secrets, and backend isolated and network-segmented?</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D17" s="6">
+        <f>IF('RAG'!$C$17="Yes","",ROUND('RAG Engine'!B55,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Do you monitor for retrieval drift/anomalies and document the system's expected behavior?</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D18" s="6">
+        <f>IF('RAG'!$C$18="Yes","",ROUND('RAG Engine'!B56,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Evidence &amp; assurance — How well the system's security is documented and tested.</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n"/>
+      <c r="D20" s="3" t="n"/>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Do you document provenance for the model AND the knowledge-base sources (AIBOM / data lineage)?</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Have you security-tested the RAG pipeline (data poisoning, indirect injection, data leakage)?</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Was that testing recent (within ~12 months) and re-run when the corpus changed?</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>RESULT</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n"/>
+      <c r="C26" s="3" t="n"/>
+      <c r="D26" s="3" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Effective Risk Score (ERS)</t>
+        </is>
+      </c>
+      <c r="C27" s="8">
+        <f>ROUND('RAG Engine'!B46,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="C28">
+        <f>IF('RAG Engine'!B46&gt;=9,"Critical",IF('RAG Engine'!B46&gt;=7,"High",IF('RAG Engine'!B46&gt;=5,"Moderate",IF('RAG Engine'!B46&gt;=3,"Low-Moderate","Low"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="C5 C6 C7 C8 C11 C12 C13 C14 C15 C16 C17 C18 C21 C22 C23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>axis</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ro-1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Ro</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D2">
+        <f>MAX(C2,IF('RAG'!$C$13="Yes",0.65,0),IF('RAG'!$C$14="Yes",0.75,0),IF('RAG'!$C$15="Yes",0.7,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ro-2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Ro</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D3">
+        <f>MAX(C3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ro-3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ro</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D4">
+        <f>MAX(C4,IF('RAG'!$C$18="Yes",0.7,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ro-4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ro</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D5">
+        <f>MAX(C5,IF('RAG'!$C$11="Yes",0.7,0),IF('RAG'!$C$15="Yes",0.65,0),IF('RAG'!$C$16="Yes",0.7,0),IF('RAG'!$C$18="Yes",0.55,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Fa-1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Fa</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D6">
+        <f>MAX(C6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Fa-2</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Fa</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D7">
+        <f>MAX(C7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Fa-3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Fa</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D8">
+        <f>MAX(C8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Fa-4</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Fa</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D9">
+        <f>MAX(C9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Tr-1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Tr</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D10">
+        <f>MAX(C10,IF('RAG'!$C$18="Yes",0.6,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Tr-2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Tr</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D11">
+        <f>MAX(C11,IF('RAG'!$C$13="Yes",0.7,0),IF('RAG'!$C$18="Yes",0.75,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Tr-3</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Tr</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D12">
+        <f>MAX(C12,IF('RAG'!$C$14="Yes",0.65,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Tr-4</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Tr</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <f>MAX(C13,IF('RAG'!$C$16="Yes",0.8,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Pr-1</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pr</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D14">
+        <f>MAX(C14,IF('RAG'!$C$12="Yes",0.7,0),IF('RAG'!$C$13="Yes",0.6,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Pr-2</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Pr</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D15">
+        <f>MAX(C15,IF('RAG'!$C$11="Yes",0.65,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Pr-3</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Pr</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D16">
+        <f>MAX(C16,IF('RAG'!$C$12="Yes",0.65,0),IF('RAG'!$C$16="Yes",0.7,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Pr-4</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Pr</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D17">
+        <f>MAX(C17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Cn-1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Cn</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D18">
+        <f>MAX(C18,IF('RAG'!$C$16="Yes",0.6,0),IF('RAG'!$C$17="Yes",0.7,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Cn-2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Cn</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D19">
+        <f>MAX(C19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Cn-3</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Cn</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D20">
+        <f>MAX(C20,IF('RAG'!$C$11="Yes",0.7,0),IF('RAG'!$C$12="Yes",0.7,0),IF('RAG'!$C$13="Yes",0.75,0),IF('RAG'!$C$17="Yes",0.65,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Cn-4</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Cn</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D21">
+        <f>MAX(C21,IF('RAG'!$C$17="Yes",0.6,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Cn-5</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Cn</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D22">
+        <f>MAX(C22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>axis averages</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Ro</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>AVERAGE(D2:D5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Fa</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>AVERAGE(D6:D9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Tr</t>
+        </is>
+      </c>
+      <c r="B26">
+        <f>AVERAGE(D10:D13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Pr</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>AVERAGE(D14:D17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Cn</t>
+        </is>
+      </c>
+      <c r="B28">
+        <f>AVERAGE(D18:D22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>IVP</t>
+        </is>
+      </c>
+      <c r="B30">
+        <f>0.25*B24+0.1*B25+0.15*B26+0.3*B27+0.2*B28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>aa</t>
+        </is>
+      </c>
+      <c r="B32">
+        <f>IF('RAG'!$C$5="Yes",0.85,0.3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>as</t>
+        </is>
+      </c>
+      <c r="B33">
+        <f>IF('RAG'!$C$6="Yes",0.85,0.3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>cp</t>
+        </is>
+      </c>
+      <c r="B34">
+        <f>IF('RAG'!$C$7="Yes",0.85,0.3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="B35">
+        <f>IF('RAG'!$C$8="Yes",0.85,0.3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>orp_avg</t>
+        </is>
+      </c>
+      <c r="B36">
+        <f>AVERAGE(B32:B35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>n_elev</t>
+        </is>
+      </c>
+      <c r="B37">
+        <f>(IF(B32&gt;0.75,1,0)+IF(B33&gt;0.75,1,0)+IF(B34&gt;0.75,1,0)+IF(B35&gt;0.75,1,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B38">
+        <f>MIN(1.75,MAX(0.75,-0.129+1.882*B36+0.05*B37))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="B40">
+        <f>IF('RAG'!$C$21="Yes",0.8,0.2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ec</t>
+        </is>
+      </c>
+      <c r="B41">
+        <f>IF('RAG'!$C$22="Yes",0.8,0.2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>tf</t>
+        </is>
+      </c>
+      <c r="B42">
+        <f>IF('RAG'!$C$22="Yes",IF('RAG'!$C$23="Yes",0.8,0.25),0.2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ACI</t>
+        </is>
+      </c>
+      <c r="B43">
+        <f>(MAX(B40,0.01)*MAX(B41,0.01)*MAX(B42,0.01))^(1/3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>aci_mod</t>
+        </is>
+      </c>
+      <c r="B44">
+        <f>1.1-0.525*B43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ERS</t>
+        </is>
+      </c>
+      <c r="B46">
+        <f>MIN(10,MAX(1.5,1.5+8.5*(1-B30)*B38*B44))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>points-you-could-save (per safeguard)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>s1</t>
+        </is>
+      </c>
+      <c r="B49">
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.25*((D2+D3+D4+MAX(D5,0.7))/4)+0.1*((D6+D7+D8+D9)/4)+0.15*((D10+D11+D12+D13)/4)+0.3*((D14+MAX(D15,0.65)+D16+D17)/4)+0.2*((D18+D19+MAX(D20,0.7)+D21+D22)/5))))*B38*B44)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>s2</t>
+        </is>
+      </c>
+      <c r="B50">
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.25*((D2+D3+D4+D5)/4)+0.1*((D6+D7+D8+D9)/4)+0.15*((D10+D11+D12+D13)/4)+0.3*((MAX(D14,0.7)+D15+MAX(D16,0.65)+D17)/4)+0.2*((D18+D19+MAX(D20,0.7)+D21+D22)/5))))*B38*B44)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>s3</t>
+        </is>
+      </c>
+      <c r="B51">
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.25*((MAX(D2,0.65)+D3+D4+D5)/4)+0.1*((D6+D7+D8+D9)/4)+0.15*((D10+MAX(D11,0.7)+D12+D13)/4)+0.3*((MAX(D14,0.6)+D15+D16+D17)/4)+0.2*((D18+D19+MAX(D20,0.75)+D21+D22)/5))))*B38*B44)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>s4</t>
+        </is>
+      </c>
+      <c r="B52">
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.25*((MAX(D2,0.75)+D3+D4+D5)/4)+0.1*((D6+D7+D8+D9)/4)+0.15*((D10+D11+MAX(D12,0.65)+D13)/4)+0.3*((D14+D15+D16+D17)/4)+0.2*((D18+D19+D20+D21+D22)/5))))*B38*B44)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>s5</t>
+        </is>
+      </c>
+      <c r="B53">
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.25*((MAX(D2,0.7)+D3+D4+MAX(D5,0.65))/4)+0.1*((D6+D7+D8+D9)/4)+0.15*((D10+D11+D12+D13)/4)+0.3*((D14+D15+D16+D17)/4)+0.2*((D18+D19+D20+D21+D22)/5))))*B38*B44)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>s6</t>
+        </is>
+      </c>
+      <c r="B54">
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.25*((D2+D3+D4+MAX(D5,0.7))/4)+0.1*((D6+D7+D8+D9)/4)+0.15*((D10+D11+D12+MAX(D13,0.8))/4)+0.3*((D14+D15+MAX(D16,0.7)+D17)/4)+0.2*((MAX(D18,0.6)+D19+D20+D21+D22)/5))))*B38*B44)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>s7</t>
+        </is>
+      </c>
+      <c r="B55">
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.25*((D2+D3+D4+D5)/4)+0.1*((D6+D7+D8+D9)/4)+0.15*((D10+D11+D12+D13)/4)+0.3*((D14+D15+D16+D17)/4)+0.2*((MAX(D18,0.7)+D19+MAX(D20,0.65)+MAX(D21,0.6)+D22)/5))))*B38*B44)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>s8</t>
+        </is>
+      </c>
+      <c r="B56">
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.25*((D2+D3+MAX(D4,0.7)+MAX(D5,0.55))/4)+0.1*((D6+D7+D8+D9)/4)+0.15*((MAX(D10,0.6)+MAX(D11,0.75)+D12+D13)/4)+0.3*((D14+D15+D16+D17)/4)+0.2*((D18+D19+D20+D21+D22)/5))))*B38*B44)))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>AITBM — Quick AI Risk Self-Assessment — Standalone LLM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Scenario: Standalone LLM. Answer Yes or No in column C; the Effective Risk Score (ERS) updates automatically. The Agentic / RAG / Standalone tabs each carry questions tailored to that architecture. Educational estimate; see the AITBM Framework Specification for assessments of record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>About your system — A few questions about your standalone model or chatbot and how it is used.</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Are the model's outputs used to drive decisions or actions automatically, without human review?</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Can the public or untrusted users send prompts or inputs to the model?</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Could a wrong output cause serious harm (financial, legal, safety, or many users)?</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Would fixing a discovered flaw be slow (retraining, fine-tuning, vendor dependency)?</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Safeguards in place — Answer Yes only for protections you have actually implemented.</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n"/>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Points you could save</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Have you adversarially trained and tested the model against manipulated inputs?</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D11" s="6">
+        <f>IF('Standalone'!$C$11="Yes","",ROUND('Standalone Engine'!B49,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Do you filter and validate both the inputs users send and the outputs the model returns?</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D12" s="6">
+        <f>IF('Standalone'!$C$12="Yes","",ROUND('Standalone Engine'!B50,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Do you have real-time detection for prompt injection and jailbreak attempts?</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D13" s="6">
+        <f>IF('Standalone'!$C$13="Yes","",ROUND('Standalone Engine'!B51,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Have you baselined the model's expected behavior/output consistency and documented it?</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D14" s="6">
+        <f>IF('Standalone'!$C$14="Yes","",ROUND('Standalone Engine'!B52,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Do you detect and block leakage of sensitive or personal data in outputs?</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D15" s="6">
+        <f>IF('Standalone'!$C$15="Yes","",ROUND('Standalone Engine'!B53,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Do you track where the model and its training data came from (lineage / AIBOM)?</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D16" s="6">
+        <f>IF('Standalone'!$C$16="Yes","",ROUND('Standalone Engine'!B54,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Do you monitor for model drift and anomalies in production?</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D17" s="6">
+        <f>IF('Standalone'!$C$17="Yes","",ROUND('Standalone Engine'!B55,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Is the model's runtime isolated and granted only least-access to surrounding systems?</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D18" s="6">
+        <f>IF('Standalone'!$C$18="Yes","",ROUND('Standalone Engine'!B56,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Evidence &amp; assurance — How well the system's security is documented and tested.</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n"/>
+      <c r="D20" s="3" t="n"/>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Do you have a model card / AIBOM documenting the model and its training-data provenance?</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Have you security-tested the model (adversarial inputs, jailbreaks, data extraction)?</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Was that testing recent (within ~12 months) and kept current with model updates?</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>RESULT</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n"/>
+      <c r="C26" s="3" t="n"/>
+      <c r="D26" s="3" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Effective Risk Score (ERS)</t>
+        </is>
+      </c>
+      <c r="C27" s="8">
+        <f>ROUND('Standalone Engine'!B46,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="C28">
+        <f>IF('Standalone Engine'!B46&gt;=9,"Critical",IF('Standalone Engine'!B46&gt;=7,"High",IF('Standalone Engine'!B46&gt;=5,"Moderate",IF('Standalone Engine'!B46&gt;=3,"Low-Moderate","Low"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Standalone LLM</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="C5 C6 C7 C8 C11 C12 C13 C14 C15 C16 C17 C18 C21 C22 C23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>axis</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ro-1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Ro</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D2">
+        <f>MAX(C2,IF('Standalone'!$C$11="Yes",0.7,0),IF('Standalone'!$C$12="Yes",0.65,0),IF('Standalone'!$C$13="Yes",0.75,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ro-2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Ro</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D3">
+        <f>MAX(C3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ro-3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ro</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D4">
+        <f>MAX(C4,IF('Standalone'!$C$14="Yes",0.7,0),IF('Standalone'!$C$17="Yes",0.65,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ro-4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ro</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D5">
+        <f>MAX(C5,IF('Standalone'!$C$11="Yes",0.65,0),IF('Standalone'!$C$16="Yes",0.7,0),IF('Standalone'!$C$17="Yes",0.55,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Fa-1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Fa</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D6">
+        <f>MAX(C6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Fa-2</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Fa</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D7">
+        <f>MAX(C7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Fa-3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Fa</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D8">
+        <f>MAX(C8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Fa-4</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Fa</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D9">
+        <f>MAX(C9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Tr-1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Tr</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D10">
+        <f>MAX(C10,IF('Standalone'!$C$14="Yes",0.6,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Tr-2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Tr</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D11">
+        <f>MAX(C11,IF('Standalone'!$C$12="Yes",0.7,0),IF('Standalone'!$C$14="Yes",0.75,0),IF('Standalone'!$C$17="Yes",0.6,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Tr-3</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Tr</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D12">
+        <f>MAX(C12,IF('Standalone'!$C$13="Yes",0.65,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Tr-4</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Tr</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <f>MAX(C13,IF('Standalone'!$C$16="Yes",0.8,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Pr-1</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pr</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D14">
+        <f>MAX(C14,IF('Standalone'!$C$12="Yes",0.6,0),IF('Standalone'!$C$15="Yes",0.7,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Pr-2</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Pr</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D15">
+        <f>MAX(C15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Pr-3</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Pr</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D16">
+        <f>MAX(C16,IF('Standalone'!$C$15="Yes",0.65,0),IF('Standalone'!$C$16="Yes",0.7,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Pr-4</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Pr</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D17">
+        <f>MAX(C17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Cn-1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Cn</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D18">
+        <f>MAX(C18,IF('Standalone'!$C$16="Yes",0.6,0),IF('Standalone'!$C$18="Yes",0.7,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Cn-2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Cn</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D19">
+        <f>MAX(C19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Cn-3</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Cn</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D20">
+        <f>MAX(C20,IF('Standalone'!$C$12="Yes",0.75,0),IF('Standalone'!$C$15="Yes",0.7,0),IF('Standalone'!$C$18="Yes",0.65,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Cn-4</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Cn</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D21">
+        <f>MAX(C21,IF('Standalone'!$C$18="Yes",0.6,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Cn-5</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Cn</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D22">
+        <f>MAX(C22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>axis averages</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Ro</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>AVERAGE(D2:D5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Fa</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>AVERAGE(D6:D9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Tr</t>
+        </is>
+      </c>
+      <c r="B26">
+        <f>AVERAGE(D10:D13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Pr</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>AVERAGE(D14:D17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Cn</t>
+        </is>
+      </c>
+      <c r="B28">
+        <f>AVERAGE(D18:D22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>IVP</t>
+        </is>
+      </c>
+      <c r="B30">
+        <f>0.25*B24+0.2*B25+0.2*B26+0.2*B27+0.15*B28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>aa</t>
+        </is>
+      </c>
+      <c r="B32">
+        <f>IF('Standalone'!$C$5="Yes",0.85,0.3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>as</t>
+        </is>
+      </c>
+      <c r="B33">
+        <f>IF('Standalone'!$C$6="Yes",0.85,0.3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>cp</t>
+        </is>
+      </c>
+      <c r="B34">
+        <f>IF('Standalone'!$C$7="Yes",0.85,0.3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="B35">
+        <f>IF('Standalone'!$C$8="Yes",0.85,0.3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>orp_avg</t>
+        </is>
+      </c>
+      <c r="B36">
+        <f>AVERAGE(B32:B35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>n_elev</t>
+        </is>
+      </c>
+      <c r="B37">
+        <f>(IF(B32&gt;0.75,1,0)+IF(B33&gt;0.75,1,0)+IF(B34&gt;0.75,1,0)+IF(B35&gt;0.75,1,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B38">
+        <f>MIN(1.75,MAX(0.75,-0.129+1.882*B36+0.05*B37))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="B40">
+        <f>IF('Standalone'!$C$21="Yes",0.8,0.2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ec</t>
+        </is>
+      </c>
+      <c r="B41">
+        <f>IF('Standalone'!$C$22="Yes",0.8,0.2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>tf</t>
+        </is>
+      </c>
+      <c r="B42">
+        <f>IF('Standalone'!$C$22="Yes",IF('Standalone'!$C$23="Yes",0.8,0.25),0.2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ACI</t>
+        </is>
+      </c>
+      <c r="B43">
+        <f>(MAX(B40,0.01)*MAX(B41,0.01)*MAX(B42,0.01))^(1/3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>aci_mod</t>
+        </is>
+      </c>
+      <c r="B44">
+        <f>1.1-0.525*B43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ERS</t>
+        </is>
+      </c>
+      <c r="B46">
+        <f>MIN(10,MAX(1.5,1.5+8.5*(1-B30)*B38*B44))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>points-you-could-save (per safeguard)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>s1</t>
+        </is>
+      </c>
+      <c r="B49">
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.25*((MAX(D2,0.7)+D3+D4+MAX(D5,0.65))/4)+0.2*((D6+D7+D8+D9)/4)+0.2*((D10+D11+D12+D13)/4)+0.2*((D14+D15+D16+D17)/4)+0.15*((D18+D19+D20+D21+D22)/5))))*B38*B44)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>s2</t>
+        </is>
+      </c>
+      <c r="B50">
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.25*((MAX(D2,0.65)+D3+D4+D5)/4)+0.2*((D6+D7+D8+D9)/4)+0.2*((D10+MAX(D11,0.7)+D12+D13)/4)+0.2*((MAX(D14,0.6)+D15+D16+D17)/4)+0.15*((D18+D19+MAX(D20,0.75)+D21+D22)/5))))*B38*B44)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>s3</t>
+        </is>
+      </c>
+      <c r="B51">
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.25*((MAX(D2,0.75)+D3+D4+D5)/4)+0.2*((D6+D7+D8+D9)/4)+0.2*((D10+D11+MAX(D12,0.65)+D13)/4)+0.2*((D14+D15+D16+D17)/4)+0.15*((D18+D19+D20+D21+D22)/5))))*B38*B44)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>s4</t>
+        </is>
+      </c>
+      <c r="B52">
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.25*((D2+D3+MAX(D4,0.7)+D5)/4)+0.2*((D6+D7+D8+D9)/4)+0.2*((MAX(D10,0.6)+MAX(D11,0.75)+D12+D13)/4)+0.2*((D14+D15+D16+D17)/4)+0.15*((D18+D19+D20+D21+D22)/5))))*B38*B44)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>s5</t>
+        </is>
+      </c>
+      <c r="B53">
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.25*((D2+D3+D4+D5)/4)+0.2*((D6+D7+D8+D9)/4)+0.2*((D10+D11+D12+D13)/4)+0.2*((MAX(D14,0.7)+D15+MAX(D16,0.65)+D17)/4)+0.15*((D18+D19+MAX(D20,0.7)+D21+D22)/5))))*B38*B44)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>s6</t>
+        </is>
+      </c>
+      <c r="B54">
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.25*((D2+D3+D4+MAX(D5,0.7))/4)+0.2*((D6+D7+D8+D9)/4)+0.2*((D10+D11+D12+MAX(D13,0.8))/4)+0.2*((D14+D15+MAX(D16,0.7)+D17)/4)+0.15*((MAX(D18,0.6)+D19+D20+D21+D22)/5))))*B38*B44)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>s7</t>
+        </is>
+      </c>
+      <c r="B55">
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.25*((D2+D3+MAX(D4,0.65)+MAX(D5,0.55))/4)+0.2*((D6+D7+D8+D9)/4)+0.2*((D10+MAX(D11,0.6)+D12+D13)/4)+0.2*((D14+D15+D16+D17)/4)+0.15*((D18+D19+D20+D21+D22)/5))))*B38*B44)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>s8</t>
+        </is>
+      </c>
+      <c r="B56">
+        <f>MAX(0,B46-MIN(10,MAX(1.5,1.5+8.5*(1-((0.25*((D2+D3+D4+D5)/4)+0.2*((D6+D7+D8+D9)/4)+0.2*((D10+D11+D12+D13)/4)+0.2*((D14+D15+D16+D17)/4)+0.15*((MAX(D18,0.7)+D19+MAX(D20,0.65)+MAX(D21,0.6)+D22)/5))))*B38*B44)))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Detailed calculator sheet to the Excel self-assessment workbook
</commit_message>
<xml_diff>
--- a/specification/AITBM_Quick_Assessment.xlsx
+++ b/specification/AITBM_Quick_Assessment.xlsx
@@ -13,6 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RAG Engine" sheetId="4" state="hidden" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standalone" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standalone Engine" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detailed" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detailed Engine" sheetId="8" state="hidden" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,8 +75,25 @@
       <color rgb="00555555"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -84,6 +103,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF2F9"/>
       </patternFill>
     </fill>
   </fills>
@@ -113,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -135,6 +159,18 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3765,4 +3801,1311 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>AITBM — Detailed ERS Calculator</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>The full calculator: pick the architecture, toggle each AIDEFEND control you have implemented (Yes/No), and set the ORP and ACI inputs (0.00 low to 1.00 high). The Effective Risk Score updates automatically. Mirrors the website's Detailed calculator; the other tabs are the plain-language scenario surveys.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>ARCHITECTURE</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Architecture (drives the axis weights)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Agentic</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>AIDEFEND CONTROLS — set Yes for each one you have implemented</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="12" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>AID-M-001</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>AI Asset Inventory &amp; Mapping</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>AID-M-002</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Data Provenance &amp; Lineage Tracking</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>AID-M-003</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Model Behavior Baseline &amp; Documentation</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>AID-M-006</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Human-in-the-Loop Control Points</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>AID-M-009</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Agent Autonomy Level Governance</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Harden</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="n"/>
+      <c r="C14" s="12" t="n"/>
+      <c r="D14" s="12" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>AID-H-001</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Adversarial Robustness Training</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>AID-H-002</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Input Sanitization &amp; Validation</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>AID-H-006</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Output Content Filtering &amp; Validation</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>AID-H-019</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Agent Permission &amp; Capability Restriction</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>AID-H-021</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Secure RAG Pipeline Implementation</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>AID-H-031</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Agentic Skill Admission Control</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>AID-H-032</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>AI-Generated Code Admission Control</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>AID-H-034</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>AI Gateway Routing Integrity</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>Detect</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="n"/>
+      <c r="C23" s="12" t="n"/>
+      <c r="D23" s="12" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>AID-D-001</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Real-Time Prompt Injection Detection</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>AID-D-002</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Model Drift &amp; Anomaly Detection</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>AID-D-003</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Sensitive Data Leakage Detection</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>AID-D-011</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Agent Behavior Monitoring &amp; Attestation</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>Isolate</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="n"/>
+      <c r="C28" s="12" t="n"/>
+      <c r="D28" s="12" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>AID-I-002</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>AI System Network Segmentation</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>AID-I-007</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Client-Side AI Execution Isolation</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>AID-I-008</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Browser Session &amp; Origin Isolation</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>Deceive</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="n"/>
+      <c r="C32" s="12" t="n"/>
+      <c r="D32" s="12" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>AID-DV-001</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>AI Honeypot &amp; Canary Deployment</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>Evict</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="n"/>
+      <c r="C34" s="12" t="n"/>
+      <c r="D34" s="12" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>AID-E-005</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Automated Threat Response &amp; Termination</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>ORP — Operational Risk Posture (0.00 low to 1.00 high)</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n"/>
+      <c r="C37" s="3" t="n"/>
+      <c r="D37" s="3" t="n"/>
+    </row>
+    <row r="38">
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>Autonomy Amplification (Aa)</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>Attack Surface Exposure (As)</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>Cascade Potential (Cp)</t>
+        </is>
+      </c>
+      <c r="C40" s="14" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>Remediation Feasibility (Rf)</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>ACI — Assurance Confidence (0.00 low to 1.00 high)</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n"/>
+      <c r="C43" s="3" t="n"/>
+      <c r="D43" s="3" t="n"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>Provenance Completeness (Pc)</t>
+        </is>
+      </c>
+      <c r="C44" s="14" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>Evaluation Coverage (Ec)</t>
+        </is>
+      </c>
+      <c r="C45" s="14" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>Temporal Freshness (Tf)</t>
+        </is>
+      </c>
+      <c r="C46" s="14" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>RESULT</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n"/>
+      <c r="C48" s="3" t="n"/>
+      <c r="D48" s="3" t="n"/>
+    </row>
+    <row r="49">
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Effective Risk Score (ERS)</t>
+        </is>
+      </c>
+      <c r="C49" s="15">
+        <f>ROUND('Detailed Engine'!B44,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="C50" s="6">
+        <f>IF('Detailed Engine'!B44&gt;=9,"Critical",IF('Detailed Engine'!B44&gt;=7,"High",IF('Detailed Engine'!B44&gt;=5,"Moderate",IF('Detailed Engine'!B44&gt;=3,"Low-Moderate","Low"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>IVP composite</t>
+        </is>
+      </c>
+      <c r="C51" s="16">
+        <f>ROUND(B35,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C52" s="16">
+        <f>ROUND(B39,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>ACI composite</t>
+        </is>
+      </c>
+      <c r="C53" s="16">
+        <f>ROUND(B41,2)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="C9 C10 C11 C12 C13 C15 C16 C17 C18 C19 C20 C21 C22 C24 C25 C26 C27 C29 C30 C31 C33 C35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Agentic,RAG,Standalone"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C38 C39 C40 C41 C44 C45 C46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>axis</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ro-1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Ro</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D2">
+        <f>MAX(C2,IF('Detailed'!$C$15="Yes",0.7,0),IF('Detailed'!$C$16="Yes",0.65,0),IF('Detailed'!$C$24="Yes",0.75,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ro-2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Ro</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D3">
+        <f>MAX(C3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ro-3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ro</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D4">
+        <f>MAX(C4,IF('Detailed'!$C$11="Yes",0.7,0),IF('Detailed'!$C$25="Yes",0.65,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ro-4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ro</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D5">
+        <f>MAX(C5,IF('Detailed'!$C$10="Yes",0.7,0),IF('Detailed'!$C$15="Yes",0.65,0),IF('Detailed'!$C$19="Yes",0.7,0),IF('Detailed'!$C$20="Yes",0.55,0),IF('Detailed'!$C$21="Yes",0.55,0),IF('Detailed'!$C$25="Yes",0.55,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Fa-1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Fa</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D6">
+        <f>MAX(C6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Fa-2</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Fa</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D7">
+        <f>MAX(C7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Fa-3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Fa</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D8">
+        <f>MAX(C8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Fa-4</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Fa</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D9">
+        <f>MAX(C9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Tr-1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Tr</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D10">
+        <f>MAX(C10,IF('Detailed'!$C$11="Yes",0.6,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Tr-2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Tr</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D11">
+        <f>MAX(C11,IF('Detailed'!$C$11="Yes",0.75,0),IF('Detailed'!$C$17="Yes",0.7,0),IF('Detailed'!$C$25="Yes",0.6,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Tr-3</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Tr</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D12">
+        <f>MAX(C12,IF('Detailed'!$C$24="Yes",0.65,0),IF('Detailed'!$C$33="Yes",0.75,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Tr-4</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Tr</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <f>MAX(C13,IF('Detailed'!$C$9="Yes",0.75,0),IF('Detailed'!$C$10="Yes",0.8,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Pr-1</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pr</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D14">
+        <f>MAX(C14,IF('Detailed'!$C$17="Yes",0.6,0),IF('Detailed'!$C$26="Yes",0.7,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Pr-2</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Pr</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D15">
+        <f>MAX(C15,IF('Detailed'!$C$19="Yes",0.65,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Pr-3</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Pr</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D16">
+        <f>MAX(C16,IF('Detailed'!$C$10="Yes",0.7,0),IF('Detailed'!$C$26="Yes",0.65,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Pr-4</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Pr</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D17">
+        <f>MAX(C17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Cn-1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Cn</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D18">
+        <f>MAX(C18,IF('Detailed'!$C$9="Yes",0.6,0),IF('Detailed'!$C$12="Yes",0.75,0),IF('Detailed'!$C$13="Yes",0.8,0),IF('Detailed'!$C$18="Yes",0.8,0),IF('Detailed'!$C$20="Yes",0.65,0),IF('Detailed'!$C$22="Yes",0.6,0),IF('Detailed'!$C$27="Yes",0.75,0),IF('Detailed'!$C$29="Yes",0.6,0),IF('Detailed'!$C$30="Yes",0.7,0),IF('Detailed'!$C$31="Yes",0.65,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Cn-2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Cn</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D19">
+        <f>MAX(C19,IF('Detailed'!$C$12="Yes",0.7,0),IF('Detailed'!$C$13="Yes",0.75,0),IF('Detailed'!$C$18="Yes",0.75,0),IF('Detailed'!$C$27="Yes",0.7,0),IF('Detailed'!$C$35="Yes",0.65,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Cn-3</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Cn</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D20">
+        <f>MAX(C20,IF('Detailed'!$C$16="Yes",0.6,0),IF('Detailed'!$C$17="Yes",0.75,0),IF('Detailed'!$C$19="Yes",0.7,0),IF('Detailed'!$C$21="Yes",0.65,0),IF('Detailed'!$C$26="Yes",0.7,0),IF('Detailed'!$C$30="Yes",0.65,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Cn-4</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Cn</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D21">
+        <f>MAX(C21,IF('Detailed'!$C$22="Yes",0.55,0),IF('Detailed'!$C$29="Yes",0.55,0),IF('Detailed'!$C$30="Yes",0.6,0),IF('Detailed'!$C$31="Yes",0.6,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Cn-5</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Cn</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D22">
+        <f>MAX(C22,IF('Detailed'!$C$13="Yes",0.7,0),IF('Detailed'!$C$18="Yes",0.7,0),IF('Detailed'!$C$27="Yes",0.8,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>axis averages</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Ro</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>AVERAGE(D2:D5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Fa</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>AVERAGE(D6:D9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Tr</t>
+        </is>
+      </c>
+      <c r="B26">
+        <f>AVERAGE(D10:D13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Pr</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>AVERAGE(D14:D17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Cn</t>
+        </is>
+      </c>
+      <c r="B28">
+        <f>AVERAGE(D18:D22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>weights (by architecture)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>w_Ro</t>
+        </is>
+      </c>
+      <c r="B30">
+        <f>IF('Detailed'!$C$5="Agentic",0.15,IF('Detailed'!$C$5="RAG",0.25,0.25))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>w_Fa</t>
+        </is>
+      </c>
+      <c r="B31">
+        <f>IF('Detailed'!$C$5="Agentic",0.1,IF('Detailed'!$C$5="RAG",0.1,0.2))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>w_Tr</t>
+        </is>
+      </c>
+      <c r="B32">
+        <f>IF('Detailed'!$C$5="Agentic",0.15,IF('Detailed'!$C$5="RAG",0.15,0.2))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>w_Pr</t>
+        </is>
+      </c>
+      <c r="B33">
+        <f>IF('Detailed'!$C$5="Agentic",0.15,IF('Detailed'!$C$5="RAG",0.3,0.2))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>w_Cn</t>
+        </is>
+      </c>
+      <c r="B34">
+        <f>IF('Detailed'!$C$5="Agentic",0.45,IF('Detailed'!$C$5="RAG",0.2,0.15))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>IVP</t>
+        </is>
+      </c>
+      <c r="B35">
+        <f>B30*B24+B31*B25+B32*B26+B33*B27+B34*B28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>orp_avg</t>
+        </is>
+      </c>
+      <c r="B37">
+        <f>('Detailed'!$C$38+'Detailed'!$C$39+'Detailed'!$C$40+'Detailed'!$C$41)/4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>n_elev</t>
+        </is>
+      </c>
+      <c r="B38">
+        <f>(IF('Detailed'!$C$38&gt;0.75,1,0)+IF('Detailed'!$C$39&gt;0.75,1,0)+IF('Detailed'!$C$40&gt;0.75,1,0)+IF('Detailed'!$C$41&gt;0.75,1,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B39">
+        <f>MIN(1.75,MAX(0.75,-0.129+1.882*B37+0.05*B38))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ACI</t>
+        </is>
+      </c>
+      <c r="B41">
+        <f>(MAX('Detailed'!$C$44,0.01)*MAX('Detailed'!$C$45,0.01)*MAX('Detailed'!$C$46,0.01))^(1/3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>aci_mod</t>
+        </is>
+      </c>
+      <c r="B42">
+        <f>1.1-0.525*B41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ERS</t>
+        </is>
+      </c>
+      <c r="B44">
+        <f>MIN(10,MAX(1.5,1.5+8.5*(1-B35)*B39*B42))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>